<commit_message>
Atualizando planilha das startups
</commit_message>
<xml_diff>
--- a/planilha_startups.xlsx
+++ b/planilha_startups.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci\Documents\Exercicios puc VS\3º Semestre\PI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C3FEF9A8-F1C6-4BEB-BADB-9DB13DF04723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{455F67ED-F946-4C9E-95B0-92D1BA892BFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="58">
   <si>
     <t>id_startup</t>
   </si>
@@ -189,12 +189,36 @@
   </si>
   <si>
     <t>https://demo.movesmart.com</t>
+  </si>
+  <si>
+    <t>valor_token</t>
+  </si>
+  <si>
+    <t>Localização</t>
+  </si>
+  <si>
+    <t>Campinas</t>
+  </si>
+  <si>
+    <t>Sumaré</t>
+  </si>
+  <si>
+    <t>Valinhos</t>
+  </si>
+  <si>
+    <t>Vinhedo</t>
+  </si>
+  <si>
+    <t>Jundiaí</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -241,7 +265,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -250,6 +274,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -555,23 +582,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="17.6640625" customWidth="1"/>
-    <col min="3" max="3" width="26.6640625" customWidth="1"/>
-    <col min="4" max="4" width="24" customWidth="1"/>
-    <col min="5" max="5" width="19" customWidth="1"/>
-    <col min="6" max="6" width="21.5546875" customWidth="1"/>
-    <col min="7" max="7" width="19.6640625" customWidth="1"/>
-    <col min="8" max="8" width="25.5546875" customWidth="1"/>
-    <col min="9" max="9" width="23.6640625" customWidth="1"/>
-    <col min="10" max="10" width="22.5546875" customWidth="1"/>
-    <col min="11" max="11" width="26" customWidth="1"/>
+    <col min="2" max="3" width="17.6640625" customWidth="1"/>
+    <col min="4" max="4" width="26.6640625" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="7" max="7" width="21.5546875" customWidth="1"/>
+    <col min="8" max="9" width="19.6640625" customWidth="1"/>
+    <col min="10" max="10" width="25.5546875" customWidth="1"/>
+    <col min="11" max="11" width="23.6640625" customWidth="1"/>
+    <col min="12" max="12" width="22.5546875" customWidth="1"/>
+    <col min="13" max="13" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -579,37 +606,43 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -617,37 +650,43 @@
         <v>38</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="2">
+      <c r="G2" s="2">
         <v>180000</v>
       </c>
-      <c r="G2" s="2">
+      <c r="H2" s="2">
         <v>70000</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="4">
+        <v>7</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -655,37 +694,43 @@
         <v>15</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="2">
+      <c r="G3" s="2">
         <v>500000</v>
       </c>
-      <c r="G3" s="2">
+      <c r="H3" s="2">
         <v>150000</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="I3" s="4">
+        <v>10</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="M3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="N3" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -693,37 +738,43 @@
         <v>23</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="2">
+      <c r="G4" s="2">
         <v>200000</v>
       </c>
-      <c r="G4" s="2">
+      <c r="H4" s="2">
         <v>80000</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="4">
+        <v>9</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="M4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -731,37 +782,43 @@
         <v>31</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="2">
+      <c r="G5" s="2">
         <v>350000</v>
       </c>
-      <c r="G5" s="2">
+      <c r="H5" s="2">
         <v>120000</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="I5" s="4">
+        <v>15</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="L5" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="M5" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="N5" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -769,37 +826,43 @@
         <v>44</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F6" s="2">
+      <c r="G6" s="2">
         <v>390000</v>
       </c>
-      <c r="G6" s="2">
+      <c r="H6" s="2">
         <v>110000</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="I6" s="4">
+        <v>12</v>
+      </c>
+      <c r="J6" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="K6" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="L6" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="K6" s="3" t="s">
+      <c r="M6" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="N6" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -812,8 +875,10 @@
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -826,8 +891,10 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -840,8 +907,10 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -854,8 +923,10 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -868,8 +939,10 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M14" s="2"/>
+      <c r="N14" s="2"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -882,14 +955,16 @@
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="K3" r:id="rId1" xr:uid="{C6EA92FD-1DDF-46E1-A215-92DC5895A16A}"/>
-    <hyperlink ref="K4" r:id="rId2" display="https://demo.healthai.com/" xr:uid="{025AD5DB-15BA-4DCB-9AFB-417E3AE0DD3A}"/>
-    <hyperlink ref="K5" r:id="rId3" display="https://demo.eduflex.com/" xr:uid="{D7F690D3-E5A4-4FFD-A461-34C5934BA8AF}"/>
-    <hyperlink ref="K2" r:id="rId4" xr:uid="{2A4B7B66-D1DC-4955-B448-7F5B47B949CF}"/>
-    <hyperlink ref="K6" r:id="rId5" xr:uid="{D1699D2A-4A30-4C5F-8489-AB6A21C451D9}"/>
+    <hyperlink ref="M3" r:id="rId1" xr:uid="{C6EA92FD-1DDF-46E1-A215-92DC5895A16A}"/>
+    <hyperlink ref="M4" r:id="rId2" display="https://demo.healthai.com/" xr:uid="{025AD5DB-15BA-4DCB-9AFB-417E3AE0DD3A}"/>
+    <hyperlink ref="M5" r:id="rId3" display="https://demo.eduflex.com/" xr:uid="{D7F690D3-E5A4-4FFD-A461-34C5934BA8AF}"/>
+    <hyperlink ref="M2" r:id="rId4" xr:uid="{2A4B7B66-D1DC-4955-B448-7F5B47B949CF}"/>
+    <hyperlink ref="M6" r:id="rId5" xr:uid="{D1699D2A-4A30-4C5F-8489-AB6A21C451D9}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>